<commit_message>
20251229: Update PCell (Donut contacts)
</commit_message>
<xml_diff>
--- a/Document/Layer_Tables/TR-1um_Drawing_Layer_DR_Table.xlsx
+++ b/Document/Layer_Tables/TR-1um_Drawing_Layer_DR_Table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/okamura/Library/CloudStorage/Dropbox/91_OpenPDK/TR-1um/Document/Layer_Tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D87137EE-18C2-144E-8875-6F96B24D8AB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0688BBF3-3E0E-AF46-8388-720C164BE291}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="840" yWindow="860" windowWidth="29400" windowHeight="18600" xr2:uid="{7F1200E8-B51D-9446-A5CE-CEA05B5231B7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="219">
   <si>
     <t>WN.W1</t>
   </si>
@@ -687,6 +687,12 @@
   </si>
   <si>
     <t>AP+AN</t>
+  </si>
+  <si>
+    <t>ER1305</t>
+  </si>
+  <si>
+    <t>M1.CL</t>
   </si>
 </sst>
 </file>
@@ -1655,7 +1661,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4478C0F2-BA21-8B4B-B7C2-220C0E7FA6A8}">
-  <dimension ref="B2:I102"/>
+  <dimension ref="B2:I103"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="19" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4.6640625" style="1" customWidth="1"/>
@@ -3472,40 +3478,40 @@
     </row>
     <row r="84" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B84" s="5" t="s">
-        <v>138</v>
+        <v>218</v>
       </c>
       <c r="C84" s="6" t="s">
-        <v>180</v>
-      </c>
-      <c r="D84" s="6"/>
+        <v>178</v>
+      </c>
+      <c r="D84" s="6" t="s">
+        <v>203</v>
+      </c>
       <c r="E84" s="5" t="s">
-        <v>152</v>
+        <v>172</v>
       </c>
       <c r="F84" s="7">
-        <v>10</v>
+        <v>1.2</v>
       </c>
       <c r="G84" s="7" t="s">
         <v>140</v>
       </c>
       <c r="H84" s="5" t="s">
-        <v>121</v>
+        <v>217</v>
       </c>
     </row>
     <row r="85" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B85" s="5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C85" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="D85" s="6" t="s">
-        <v>180</v>
-      </c>
+      <c r="D85" s="6"/>
       <c r="E85" s="5" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F85" s="7">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="G85" s="7" t="s">
         <v>140</v>
@@ -3515,257 +3521,263 @@
       </c>
     </row>
     <row r="86" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B86" s="10" t="s">
-        <v>82</v>
-      </c>
-      <c r="C86" s="11" t="s">
-        <v>181</v>
-      </c>
-      <c r="D86" s="11"/>
-      <c r="E86" s="10" t="s">
-        <v>191</v>
-      </c>
-      <c r="F86" s="12">
-        <v>1.4</v>
-      </c>
-      <c r="G86" s="12" t="s">
-        <v>140</v>
-      </c>
-      <c r="H86" s="10" t="s">
-        <v>115</v>
+      <c r="B86" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="C86" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="D86" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="E86" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="F86" s="7">
+        <v>2</v>
+      </c>
+      <c r="G86" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="H86" s="5" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="87" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B87" s="10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C87" s="11" t="s">
         <v>181</v>
       </c>
-      <c r="D87" s="11" t="s">
-        <v>181</v>
-      </c>
+      <c r="D87" s="11"/>
       <c r="E87" s="10" t="s">
-        <v>153</v>
+        <v>191</v>
       </c>
       <c r="F87" s="12">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="G87" s="12" t="s">
         <v>140</v>
       </c>
       <c r="H87" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="88" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B88" s="10" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C88" s="11" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D88" s="11" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="E88" s="10" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="F88" s="12">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="G88" s="12" t="s">
         <v>140</v>
       </c>
       <c r="H88" s="10" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
     </row>
     <row r="89" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B89" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C89" s="11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D89" s="11" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="E89" s="10" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="F89" s="12">
-        <v>1.2</v>
+        <v>1</v>
       </c>
       <c r="G89" s="12" t="s">
         <v>140</v>
       </c>
       <c r="H89" s="10" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="90" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B90" s="10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C90" s="11" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D90" s="11" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E90" s="10" t="s">
         <v>153</v>
       </c>
       <c r="F90" s="12">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="G90" s="12" t="s">
         <v>140</v>
       </c>
       <c r="H90" s="10" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="91" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B91" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C91" s="11" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D91" s="11" t="s">
-        <v>203</v>
+        <v>169</v>
       </c>
       <c r="E91" s="10" t="s">
         <v>153</v>
       </c>
       <c r="F91" s="12">
+        <v>1</v>
+      </c>
+      <c r="G91" s="12" t="s">
+        <v>140</v>
+      </c>
+      <c r="H91" s="10" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="92" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B92" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="C92" s="11" t="s">
+        <v>185</v>
+      </c>
+      <c r="D92" s="11" t="s">
+        <v>203</v>
+      </c>
+      <c r="E92" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="F92" s="12">
         <v>1.4</v>
       </c>
-      <c r="G91" s="12" t="s">
-        <v>140</v>
-      </c>
-      <c r="H91" s="10" t="s">
+      <c r="G92" s="12" t="s">
+        <v>140</v>
+      </c>
+      <c r="H92" s="10" t="s">
         <v>124</v>
-      </c>
-    </row>
-    <row r="92" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B92" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="C92" s="6" t="s">
-        <v>186</v>
-      </c>
-      <c r="D92" s="6"/>
-      <c r="E92" s="5" t="s">
-        <v>152</v>
-      </c>
-      <c r="F92" s="7">
-        <v>3</v>
-      </c>
-      <c r="G92" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="H92" s="5" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="93" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B93" s="5" t="s">
-        <v>135</v>
+        <v>88</v>
       </c>
       <c r="C93" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="D93" s="6" t="s">
-        <v>186</v>
-      </c>
+      <c r="D93" s="6"/>
       <c r="E93" s="5" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F93" s="7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G93" s="7" t="s">
         <v>140</v>
       </c>
       <c r="H93" s="5" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="94" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B94" s="5" t="s">
-        <v>147</v>
+        <v>135</v>
       </c>
       <c r="C94" s="6" t="s">
         <v>186</v>
       </c>
       <c r="D94" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="E94" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="F94" s="7">
+        <v>2</v>
+      </c>
+      <c r="G94" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="H94" s="5" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="95" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B95" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="C95" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="D95" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="E94" s="5" t="s">
+      <c r="E95" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="F94" s="7">
+      <c r="F95" s="7">
         <v>1</v>
       </c>
-      <c r="G94" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="H94" s="5" t="s">
+      <c r="G95" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="H95" s="5" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="95" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B95" s="16" t="s">
+    <row r="96" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B96" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="C95" s="17" t="s">
+      <c r="C96" s="17" t="s">
         <v>192</v>
       </c>
-      <c r="D95" s="17" t="s">
+      <c r="D96" s="17" t="s">
         <v>193</v>
       </c>
-      <c r="E95" s="18" t="s">
+      <c r="E96" s="18" t="s">
         <v>151</v>
       </c>
-      <c r="F95" s="19" t="s">
+      <c r="F96" s="19" t="s">
         <v>187</v>
       </c>
-      <c r="G95" s="19" t="s">
+      <c r="G96" s="19" t="s">
         <v>137</v>
       </c>
-      <c r="H95" s="18" t="s">
+      <c r="H96" s="18" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="96" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B96" s="5" t="s">
-        <v>204</v>
-      </c>
-      <c r="C96" s="6" t="s">
-        <v>188</v>
-      </c>
-      <c r="D96" s="6" t="s">
-        <v>206</v>
-      </c>
-      <c r="E96" s="5" t="s">
-        <v>205</v>
-      </c>
-      <c r="F96" s="7"/>
-      <c r="G96" s="7"/>
-      <c r="H96" s="5"/>
     </row>
     <row r="97" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B97" s="5" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="C97" s="6" t="s">
         <v>188</v>
       </c>
       <c r="D97" s="6" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="E97" s="5" t="s">
         <v>205</v>
@@ -3776,13 +3788,13 @@
     </row>
     <row r="98" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B98" s="5" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="C98" s="6" t="s">
-        <v>169</v>
+        <v>188</v>
       </c>
       <c r="D98" s="6" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="E98" s="5" t="s">
         <v>205</v>
@@ -3793,13 +3805,13 @@
     </row>
     <row r="99" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B99" s="5" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C99" s="6" t="s">
         <v>169</v>
       </c>
       <c r="D99" s="6" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="E99" s="5" t="s">
         <v>205</v>
@@ -3810,13 +3822,13 @@
     </row>
     <row r="100" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B100" s="5" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="C100" s="6" t="s">
         <v>169</v>
       </c>
       <c r="D100" s="6" t="s">
-        <v>178</v>
+        <v>211</v>
       </c>
       <c r="E100" s="5" t="s">
         <v>205</v>
@@ -3827,10 +3839,10 @@
     </row>
     <row r="101" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B101" s="5" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C101" s="6" t="s">
-        <v>181</v>
+        <v>169</v>
       </c>
       <c r="D101" s="6" t="s">
         <v>178</v>
@@ -3844,13 +3856,13 @@
     </row>
     <row r="102" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B102" s="5" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C102" s="6" t="s">
         <v>181</v>
       </c>
       <c r="D102" s="6" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="E102" s="5" t="s">
         <v>205</v>
@@ -3858,6 +3870,23 @@
       <c r="F102" s="7"/>
       <c r="G102" s="7"/>
       <c r="H102" s="5"/>
+    </row>
+    <row r="103" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B103" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="C103" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="D103" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="E103" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="F103" s="7"/>
+      <c r="G103" s="7"/>
+      <c r="H103" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
20251230: DRC script revised.
</commit_message>
<xml_diff>
--- a/Document/Layer_Tables/TR-1um_Drawing_Layer_DR_Table.xlsx
+++ b/Document/Layer_Tables/TR-1um_Drawing_Layer_DR_Table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/okamura/Library/CloudStorage/Dropbox/91_OpenPDK/TR-1um/Document/Layer_Tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D75F27A-B787-1E49-A655-578E149F00E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA2B3D30-4CCF-FF43-BEA6-D8967F05A87A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="12080" yWindow="2880" windowWidth="29420" windowHeight="18600" xr2:uid="{7F1200E8-B51D-9446-A5CE-CEA05B5231B7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="494" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="498" uniqueCount="227">
   <si>
     <t>WN.W1</t>
   </si>
@@ -119,9 +119,6 @@
     <t>ERWLMP03</t>
   </si>
   <si>
-    <t>ERRR07</t>
-  </si>
-  <si>
     <t>ERWLRR02</t>
   </si>
   <si>
@@ -656,9 +653,6 @@
     <t>AP+AC</t>
   </si>
   <si>
-    <t>PR</t>
-  </si>
-  <si>
     <t>AR/PR related</t>
   </si>
   <si>
@@ -705,6 +699,24 @@
   </si>
   <si>
     <t>PO-AN</t>
+  </si>
+  <si>
+    <t>RS</t>
+  </si>
+  <si>
+    <t>RR</t>
+  </si>
+  <si>
+    <t>RR(W)</t>
+  </si>
+  <si>
+    <t>RS(W)</t>
+  </si>
+  <si>
+    <t>RS(L)</t>
+  </si>
+  <si>
+    <t>RR(L)</t>
   </si>
 </sst>
 </file>
@@ -1727,10 +1739,10 @@
   <sheetData>
     <row r="2" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B2" s="22" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D2" s="23"/>
       <c r="E2" s="22"/>
@@ -1740,39 +1752,39 @@
     </row>
     <row r="3" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C3" s="19" t="s">
+        <v>175</v>
+      </c>
+      <c r="D3" s="19" t="s">
+        <v>176</v>
+      </c>
+      <c r="E3" s="20" t="s">
+        <v>143</v>
+      </c>
+      <c r="F3" s="21" t="s">
+        <v>170</v>
+      </c>
+      <c r="G3" s="21" t="s">
+        <v>132</v>
+      </c>
+      <c r="H3" s="20" t="s">
         <v>88</v>
-      </c>
-      <c r="C3" s="19" t="s">
-        <v>176</v>
-      </c>
-      <c r="D3" s="19" t="s">
-        <v>177</v>
-      </c>
-      <c r="E3" s="20" t="s">
-        <v>144</v>
-      </c>
-      <c r="F3" s="21" t="s">
-        <v>171</v>
-      </c>
-      <c r="G3" s="21" t="s">
-        <v>133</v>
-      </c>
-      <c r="H3" s="20" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="4" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="5" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F4" s="6">
         <v>0</v>
@@ -1782,16 +1794,16 @@
     </row>
     <row r="5" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="5" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F5" s="6">
         <v>0</v>
@@ -1801,16 +1813,16 @@
     </row>
     <row r="6" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="5" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F6" s="6">
         <v>0</v>
@@ -1820,16 +1832,16 @@
     </row>
     <row r="7" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F7" s="6">
         <v>0</v>
@@ -1839,16 +1851,16 @@
     </row>
     <row r="8" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F8" s="6">
         <v>0</v>
@@ -1858,16 +1870,16 @@
     </row>
     <row r="9" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="5" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C9" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="D9" s="11" t="s">
         <v>169</v>
       </c>
-      <c r="D9" s="11" t="s">
-        <v>170</v>
-      </c>
       <c r="E9" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F9" s="6">
         <v>0</v>
@@ -1877,10 +1889,10 @@
     </row>
     <row r="10" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B10" s="22" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D10" s="23"/>
       <c r="E10" s="22"/>
@@ -1890,25 +1902,25 @@
     </row>
     <row r="11" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="H11" s="1" t="s">
         <v>88</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="12" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
@@ -1916,11 +1928,11 @@
         <v>0</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D12" s="11"/>
       <c r="E12" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F12" s="6">
         <v>8</v>
@@ -1935,13 +1947,13 @@
         <v>1</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F13" s="6">
         <v>12</v>
@@ -1956,13 +1968,13 @@
         <v>2</v>
       </c>
       <c r="C14" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="D14" s="12" t="s">
         <v>172</v>
       </c>
-      <c r="D14" s="12" t="s">
-        <v>173</v>
-      </c>
       <c r="E14" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F14" s="6">
         <v>9.5</v>
@@ -1977,13 +1989,13 @@
         <v>3</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D15" s="12" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F15" s="6">
         <v>12</v>
@@ -1998,13 +2010,13 @@
         <v>4</v>
       </c>
       <c r="C16" s="12" t="s">
+        <v>172</v>
+      </c>
+      <c r="D16" s="12" t="s">
         <v>173</v>
       </c>
-      <c r="D16" s="12" t="s">
-        <v>174</v>
-      </c>
       <c r="E16" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F16" s="6">
         <v>9.5</v>
@@ -2019,13 +2031,13 @@
         <v>5</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F17" s="6">
         <v>8</v>
@@ -2040,13 +2052,13 @@
         <v>6</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F18" s="6">
         <v>12</v>
@@ -2061,13 +2073,13 @@
         <v>7</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F19" s="6">
         <v>5</v>
@@ -2082,13 +2094,13 @@
         <v>8</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F20" s="6">
         <v>10</v>
@@ -2100,82 +2112,82 @@
     </row>
     <row r="21" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B21" s="8" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>149</v>
-      </c>
-      <c r="D21" s="13"/>
+        <v>148</v>
+      </c>
+      <c r="D21" s="13" t="s">
+        <v>161</v>
+      </c>
       <c r="E21" s="8" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F21" s="9">
-        <v>2.8</v>
-      </c>
-      <c r="G21" s="9">
-        <v>20</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="G21" s="9"/>
       <c r="H21" s="8" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="22" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B22" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>149</v>
+        <v>161</v>
       </c>
       <c r="D22" s="13" t="s">
-        <v>162</v>
+        <v>172</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F22" s="9">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="G22" s="9"/>
       <c r="H22" s="8" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="23" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B23" s="8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F23" s="9">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G23" s="9"/>
       <c r="H23" s="8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="24" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="D24" s="13" t="s">
-        <v>173</v>
+        <v>154</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="F24" s="9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G24" s="9"/>
       <c r="H24" s="8" t="s">
@@ -2183,24 +2195,24 @@
       </c>
     </row>
     <row r="25" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="C25" s="13" t="s">
-        <v>162</v>
-      </c>
-      <c r="D25" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="E25" s="8" t="s">
+      <c r="B25" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C25" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="D25" s="11"/>
+      <c r="E25" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="F25" s="9">
-        <v>4</v>
-      </c>
-      <c r="G25" s="9"/>
-      <c r="H25" s="8" t="s">
-        <v>31</v>
+      <c r="F25" s="6">
+        <v>28.5</v>
+      </c>
+      <c r="G25" s="6">
+        <v>120</v>
+      </c>
+      <c r="H25" s="5" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="26" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
@@ -2208,40 +2220,40 @@
         <v>32</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>150</v>
-      </c>
-      <c r="D26" s="11"/>
+        <v>149</v>
+      </c>
+      <c r="D26" s="11" t="s">
+        <v>149</v>
+      </c>
       <c r="E26" s="5" t="s">
-        <v>147</v>
-      </c>
-      <c r="F26" s="6">
-        <v>28.5</v>
-      </c>
-      <c r="G26" s="6">
-        <v>120</v>
-      </c>
-      <c r="H26" s="5" t="s">
-        <v>125</v>
-      </c>
+        <v>145</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="G26" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="H26" s="5"/>
     </row>
     <row r="27" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B27" s="5" t="s">
         <v>33</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D27" s="11" t="s">
-        <v>150</v>
+        <v>173</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G27" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="H27" s="5"/>
     </row>
@@ -2250,37 +2262,37 @@
         <v>34</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="F28" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="G28" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="H28" s="5"/>
+        <v>147</v>
+      </c>
+      <c r="F28" s="6">
+        <v>3</v>
+      </c>
+      <c r="G28" s="6"/>
+      <c r="H28" s="5" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="29" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="5" t="s">
         <v>35</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>174</v>
+        <v>154</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="F29" s="6">
-        <v>3</v>
+        <v>2.8</v>
       </c>
       <c r="G29" s="6"/>
       <c r="H29" s="5" t="s">
@@ -2289,78 +2301,76 @@
     </row>
     <row r="30" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="5" t="s">
-        <v>36</v>
+        <v>90</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D30" s="11" t="s">
-        <v>155</v>
+        <v>215</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>146</v>
+        <v>179</v>
       </c>
       <c r="F30" s="6">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="G30" s="6"/>
-      <c r="H30" s="5" t="s">
+      <c r="H30" s="5"/>
+    </row>
+    <row r="31" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B31" s="22" t="s">
+        <v>203</v>
+      </c>
+      <c r="C31" s="18" t="s">
+        <v>198</v>
+      </c>
+      <c r="D31" s="23"/>
+      <c r="E31" s="22"/>
+      <c r="F31" s="24"/>
+      <c r="G31" s="24"/>
+      <c r="H31" s="22"/>
+    </row>
+    <row r="32" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B32" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="G32" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="33" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B33" s="8" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="31" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B31" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="C31" s="11" t="s">
-        <v>150</v>
-      </c>
-      <c r="D31" s="11" t="s">
-        <v>217</v>
-      </c>
-      <c r="E31" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="F31" s="6">
-        <v>0</v>
-      </c>
-      <c r="G31" s="6"/>
-      <c r="H31" s="5"/>
-    </row>
-    <row r="32" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B32" s="22" t="s">
-        <v>204</v>
-      </c>
-      <c r="C32" s="18" t="s">
-        <v>199</v>
-      </c>
-      <c r="D32" s="23"/>
-      <c r="E32" s="22"/>
-      <c r="F32" s="24"/>
-      <c r="G32" s="24"/>
-      <c r="H32" s="22"/>
-    </row>
-    <row r="33" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B33" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="E33" s="1" t="s">
+      <c r="C33" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="D33" s="13"/>
+      <c r="E33" s="8" t="s">
         <v>144</v>
       </c>
-      <c r="F33" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="G33" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="H33" s="1" t="s">
-        <v>89</v>
+      <c r="F33" s="9">
+        <v>1.4</v>
+      </c>
+      <c r="G33" s="9"/>
+      <c r="H33" s="8" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="34" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
@@ -2368,9 +2378,11 @@
         <v>39</v>
       </c>
       <c r="C34" s="13" t="s">
-        <v>152</v>
-      </c>
-      <c r="D34" s="13"/>
+        <v>151</v>
+      </c>
+      <c r="D34" s="13" t="s">
+        <v>151</v>
+      </c>
       <c r="E34" s="8" t="s">
         <v>145</v>
       </c>
@@ -2379,7 +2391,7 @@
       </c>
       <c r="G34" s="9"/>
       <c r="H34" s="8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="35" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
@@ -2387,20 +2399,20 @@
         <v>40</v>
       </c>
       <c r="C35" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D35" s="13" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F35" s="9">
-        <v>1.4</v>
+        <v>2.8</v>
       </c>
       <c r="G35" s="9"/>
       <c r="H35" s="8" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="36" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
@@ -2411,124 +2423,124 @@
         <v>152</v>
       </c>
       <c r="D36" s="13" t="s">
-        <v>155</v>
+        <v>206</v>
       </c>
       <c r="E36" s="8" t="s">
         <v>146</v>
       </c>
       <c r="F36" s="9">
-        <v>2.8</v>
-      </c>
-      <c r="G36" s="9"/>
+        <v>3.4</v>
+      </c>
+      <c r="G36" s="9">
+        <v>60</v>
+      </c>
       <c r="H36" s="8" t="s">
-        <v>58</v>
+        <v>124</v>
       </c>
     </row>
     <row r="37" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B37" s="8" t="s">
-        <v>42</v>
+        <v>136</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D37" s="13" t="s">
-        <v>208</v>
+        <v>220</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="F37" s="9">
-        <v>3.4</v>
+        <v>1</v>
       </c>
       <c r="G37" s="9">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="H37" s="8" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="38" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B38" s="8" t="s">
-        <v>137</v>
+        <v>16</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D38" s="13" t="s">
-        <v>222</v>
+        <v>171</v>
       </c>
       <c r="E38" s="8" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="F38" s="9">
-        <v>1</v>
-      </c>
-      <c r="G38" s="9">
-        <v>30</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="G38" s="9"/>
       <c r="H38" s="8" t="s">
-        <v>125</v>
+        <v>25</v>
       </c>
     </row>
     <row r="39" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B39" s="8" t="s">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>152</v>
-      </c>
-      <c r="D39" s="13" t="s">
-        <v>172</v>
-      </c>
+        <v>153</v>
+      </c>
+      <c r="D39" s="13"/>
       <c r="E39" s="8" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="F39" s="9">
-        <v>7</v>
+        <v>2.8</v>
       </c>
       <c r="G39" s="9"/>
-      <c r="H39" s="8" t="s">
-        <v>25</v>
-      </c>
+      <c r="H39" s="8"/>
     </row>
     <row r="40" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B40" s="8" t="s">
         <v>47</v>
       </c>
       <c r="C40" s="13" t="s">
-        <v>154</v>
-      </c>
-      <c r="D40" s="13"/>
+        <v>153</v>
+      </c>
+      <c r="D40" s="13" t="s">
+        <v>153</v>
+      </c>
       <c r="E40" s="8" t="s">
         <v>145</v>
       </c>
-      <c r="F40" s="9">
-        <v>2.8</v>
-      </c>
-      <c r="G40" s="9"/>
-      <c r="H40" s="8"/>
+      <c r="F40" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="G40" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="H40" s="8" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="41" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B41" s="8" t="s">
         <v>48</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D41" s="13" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>146</v>
-      </c>
-      <c r="F41" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="G41" s="9" t="s">
-        <v>59</v>
-      </c>
+        <v>145</v>
+      </c>
+      <c r="F41" s="9">
+        <v>2.8</v>
+      </c>
+      <c r="G41" s="9"/>
       <c r="H41" s="8" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
     </row>
     <row r="42" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
@@ -2536,13 +2548,13 @@
         <v>49</v>
       </c>
       <c r="C42" s="13" t="s">
+        <v>153</v>
+      </c>
+      <c r="D42" s="13" t="s">
         <v>154</v>
       </c>
-      <c r="D42" s="13" t="s">
-        <v>152</v>
-      </c>
       <c r="E42" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F42" s="9">
         <v>2.8</v>
@@ -2553,24 +2565,22 @@
       </c>
     </row>
     <row r="43" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B43" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="C43" s="13" t="s">
+      <c r="B43" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C43" s="11" t="s">
         <v>154</v>
       </c>
-      <c r="D43" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="E43" s="8" t="s">
-        <v>146</v>
-      </c>
-      <c r="F43" s="9">
-        <v>2.8</v>
-      </c>
-      <c r="G43" s="9"/>
-      <c r="H43" s="8" t="s">
-        <v>55</v>
+      <c r="D43" s="11"/>
+      <c r="E43" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="F43" s="6">
+        <v>1.4</v>
+      </c>
+      <c r="G43" s="6"/>
+      <c r="H43" s="5" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="44" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
@@ -2578,9 +2588,11 @@
         <v>43</v>
       </c>
       <c r="C44" s="11" t="s">
-        <v>155</v>
-      </c>
-      <c r="D44" s="11"/>
+        <v>154</v>
+      </c>
+      <c r="D44" s="11" t="s">
+        <v>154</v>
+      </c>
       <c r="E44" s="5" t="s">
         <v>145</v>
       </c>
@@ -2589,156 +2601,156 @@
       </c>
       <c r="G44" s="6"/>
       <c r="H44" s="5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="45" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B45" s="5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C45" s="11" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D45" s="11" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F45" s="6">
-        <v>1.4</v>
+        <v>2.8</v>
       </c>
       <c r="G45" s="6"/>
       <c r="H45" s="5" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="46" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B46" s="5" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C46" s="11" t="s">
         <v>155</v>
       </c>
       <c r="D46" s="11" t="s">
-        <v>152</v>
+        <v>207</v>
       </c>
       <c r="E46" s="5" t="s">
         <v>146</v>
       </c>
       <c r="F46" s="6">
-        <v>2.8</v>
-      </c>
-      <c r="G46" s="6"/>
+        <v>3.4</v>
+      </c>
+      <c r="G46" s="6">
+        <v>60</v>
+      </c>
       <c r="H46" s="5" t="s">
-        <v>60</v>
+        <v>124</v>
       </c>
     </row>
     <row r="47" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B47" s="5" t="s">
-        <v>45</v>
+        <v>140</v>
       </c>
       <c r="C47" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D47" s="11" t="s">
-        <v>209</v>
+        <v>220</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="F47" s="6">
-        <v>3.4</v>
+        <v>1</v>
       </c>
       <c r="G47" s="6">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="H47" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="48" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B48" s="5" t="s">
-        <v>141</v>
+        <v>17</v>
       </c>
       <c r="C48" s="11" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="D48" s="11" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="F48" s="6">
-        <v>1</v>
-      </c>
-      <c r="G48" s="6">
-        <v>30</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="G48" s="6"/>
       <c r="H48" s="5" t="s">
-        <v>125</v>
+        <v>26</v>
       </c>
     </row>
     <row r="49" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B49" s="5" t="s">
-        <v>17</v>
+        <v>177</v>
       </c>
       <c r="C49" s="11" t="s">
-        <v>155</v>
-      </c>
-      <c r="D49" s="11" t="s">
-        <v>220</v>
-      </c>
+        <v>156</v>
+      </c>
+      <c r="D49" s="11"/>
       <c r="E49" s="5" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="F49" s="6">
-        <v>5</v>
+        <v>2.8</v>
       </c>
       <c r="G49" s="6"/>
-      <c r="H49" s="5" t="s">
-        <v>26</v>
-      </c>
+      <c r="H49" s="5"/>
     </row>
     <row r="50" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B50" s="5" t="s">
-        <v>178</v>
+        <v>50</v>
       </c>
       <c r="C50" s="11" t="s">
-        <v>157</v>
-      </c>
-      <c r="D50" s="11"/>
+        <v>156</v>
+      </c>
+      <c r="D50" s="11" t="s">
+        <v>156</v>
+      </c>
       <c r="E50" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="F50" s="6">
-        <v>2.8</v>
-      </c>
-      <c r="G50" s="6"/>
-      <c r="H50" s="5"/>
+      <c r="F50" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="G50" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="H50" s="5" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="51" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B51" s="5" t="s">
         <v>51</v>
       </c>
       <c r="C51" s="11" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D51" s="11" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="F51" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="G51" s="6" t="s">
-        <v>59</v>
-      </c>
+        <v>145</v>
+      </c>
+      <c r="F51" s="6">
+        <v>2.8</v>
+      </c>
+      <c r="G51" s="6"/>
       <c r="H51" s="5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="52" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
@@ -2746,13 +2758,13 @@
         <v>52</v>
       </c>
       <c r="C52" s="11" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D52" s="11" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F52" s="6">
         <v>2.8</v>
@@ -2762,61 +2774,61 @@
         <v>61</v>
       </c>
     </row>
-    <row r="53" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B53" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="C53" s="11" t="s">
+    <row r="53" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B53" s="22" t="s">
+        <v>203</v>
+      </c>
+      <c r="C53" s="18" t="s">
+        <v>199</v>
+      </c>
+      <c r="D53" s="23"/>
+      <c r="E53" s="22"/>
+      <c r="F53" s="24"/>
+      <c r="G53" s="24"/>
+      <c r="H53" s="22"/>
+    </row>
+    <row r="54" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B54" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="E54" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="F54" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="G54" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="H54" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="55" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B55" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="C55" s="13" t="s">
         <v>157</v>
       </c>
-      <c r="D53" s="11" t="s">
-        <v>155</v>
-      </c>
-      <c r="E53" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="F53" s="6">
-        <v>2.8</v>
-      </c>
-      <c r="G53" s="6"/>
-      <c r="H53" s="5" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="54" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B54" s="22" t="s">
-        <v>204</v>
-      </c>
-      <c r="C54" s="18" t="s">
-        <v>200</v>
-      </c>
-      <c r="D54" s="23"/>
-      <c r="E54" s="22"/>
-      <c r="F54" s="24"/>
-      <c r="G54" s="24"/>
-      <c r="H54" s="22"/>
-    </row>
-    <row r="55" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B55" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="C55" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="D55" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="E55" s="1" t="s">
+      <c r="D55" s="13"/>
+      <c r="E55" s="8" t="s">
         <v>144</v>
       </c>
-      <c r="F55" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="G55" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="H55" s="1" t="s">
-        <v>89</v>
+      <c r="F55" s="9">
+        <v>1</v>
+      </c>
+      <c r="G55" s="9">
+        <v>30</v>
+      </c>
+      <c r="H55" s="8" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="56" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
@@ -2824,18 +2836,18 @@
         <v>63</v>
       </c>
       <c r="C56" s="13" t="s">
-        <v>158</v>
-      </c>
-      <c r="D56" s="13"/>
+        <v>157</v>
+      </c>
+      <c r="D56" s="13" t="s">
+        <v>157</v>
+      </c>
       <c r="E56" s="8" t="s">
         <v>145</v>
       </c>
       <c r="F56" s="9">
-        <v>1</v>
-      </c>
-      <c r="G56" s="9">
-        <v>30</v>
-      </c>
+        <v>1.2</v>
+      </c>
+      <c r="G56" s="9"/>
       <c r="H56" s="8" t="s">
         <v>92</v>
       </c>
@@ -2845,16 +2857,16 @@
         <v>64</v>
       </c>
       <c r="C57" s="13" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D57" s="13" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="E57" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F57" s="9">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="G57" s="9"/>
       <c r="H57" s="8" t="s">
@@ -2866,13 +2878,13 @@
         <v>65</v>
       </c>
       <c r="C58" s="13" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D58" s="13" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E58" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F58" s="9">
         <v>0.4</v>
@@ -2884,65 +2896,63 @@
     </row>
     <row r="59" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B59" s="8" t="s">
-        <v>66</v>
+        <v>211</v>
       </c>
       <c r="C59" s="13" t="s">
-        <v>158</v>
+        <v>208</v>
       </c>
       <c r="D59" s="13" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E59" s="8" t="s">
-        <v>146</v>
+        <v>210</v>
       </c>
       <c r="F59" s="9">
-        <v>0.4</v>
+        <v>1.2</v>
       </c>
       <c r="G59" s="9"/>
       <c r="H59" s="8" t="s">
-        <v>95</v>
+        <v>213</v>
       </c>
     </row>
     <row r="60" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B60" s="8" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C60" s="13" t="s">
+        <v>209</v>
+      </c>
+      <c r="D60" s="13" t="s">
+        <v>157</v>
+      </c>
+      <c r="E60" s="8" t="s">
         <v>210</v>
-      </c>
-      <c r="D60" s="13" t="s">
-        <v>158</v>
-      </c>
-      <c r="E60" s="8" t="s">
-        <v>212</v>
       </c>
       <c r="F60" s="9">
         <v>1.2</v>
       </c>
       <c r="G60" s="9"/>
       <c r="H60" s="8" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="61" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B61" s="8" t="s">
-        <v>214</v>
-      </c>
-      <c r="C61" s="13" t="s">
-        <v>211</v>
-      </c>
-      <c r="D61" s="13" t="s">
+      <c r="B61" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="C61" s="11" t="s">
         <v>158</v>
       </c>
-      <c r="E61" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="F61" s="9">
-        <v>1.2</v>
-      </c>
-      <c r="G61" s="9"/>
-      <c r="H61" s="8" t="s">
-        <v>216</v>
+      <c r="D61" s="11"/>
+      <c r="E61" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="F61" s="6">
+        <v>1</v>
+      </c>
+      <c r="G61" s="6"/>
+      <c r="H61" s="5" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="62" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
@@ -2950,9 +2960,11 @@
         <v>67</v>
       </c>
       <c r="C62" s="11" t="s">
-        <v>159</v>
-      </c>
-      <c r="D62" s="11"/>
+        <v>158</v>
+      </c>
+      <c r="D62" s="11" t="s">
+        <v>158</v>
+      </c>
       <c r="E62" s="5" t="s">
         <v>145</v>
       </c>
@@ -2971,14 +2983,12 @@
       <c r="C63" s="11" t="s">
         <v>159</v>
       </c>
-      <c r="D63" s="11" t="s">
-        <v>159</v>
-      </c>
+      <c r="D63" s="11"/>
       <c r="E63" s="5" t="s">
-        <v>146</v>
+        <v>174</v>
       </c>
       <c r="F63" s="6">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="G63" s="6"/>
       <c r="H63" s="5" t="s">
@@ -2987,56 +2997,58 @@
     </row>
     <row r="64" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B64" s="5" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C64" s="11" t="s">
-        <v>160</v>
-      </c>
-      <c r="D64" s="11"/>
+        <v>159</v>
+      </c>
+      <c r="D64" s="11" t="s">
+        <v>190</v>
+      </c>
       <c r="E64" s="5" t="s">
-        <v>175</v>
+        <v>147</v>
       </c>
       <c r="F64" s="6">
         <v>1.2</v>
       </c>
       <c r="G64" s="6"/>
       <c r="H64" s="5" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="65" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B65" s="5" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="C65" s="11" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D65" s="11" t="s">
-        <v>191</v>
+        <v>151</v>
       </c>
       <c r="E65" s="5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F65" s="6">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="G65" s="6"/>
       <c r="H65" s="5" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
     </row>
     <row r="66" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B66" s="5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C66" s="11" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D66" s="11" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E66" s="5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F66" s="6">
         <v>0.8</v>
@@ -3048,19 +3060,19 @@
     </row>
     <row r="67" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B67" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C67" s="11" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D67" s="11" t="s">
-        <v>155</v>
+        <v>178</v>
       </c>
       <c r="E67" s="5" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="F67" s="6">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="G67" s="6"/>
       <c r="H67" s="5" t="s">
@@ -3072,89 +3084,93 @@
         <v>72</v>
       </c>
       <c r="C68" s="11" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D68" s="11" t="s">
-        <v>179</v>
+        <v>157</v>
       </c>
       <c r="E68" s="5" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F68" s="6">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="G68" s="6"/>
       <c r="H68" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="69" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B69" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="C69" s="11" t="s">
-        <v>159</v>
-      </c>
-      <c r="D69" s="11" t="s">
-        <v>158</v>
-      </c>
-      <c r="E69" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="F69" s="6">
-        <v>0.8</v>
-      </c>
-      <c r="G69" s="6"/>
-      <c r="H69" s="5" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="70" spans="2:8" ht="20" x14ac:dyDescent="0.2">
-      <c r="B70" s="22" t="s">
-        <v>204</v>
-      </c>
-      <c r="C70" s="18" t="s">
-        <v>207</v>
-      </c>
-      <c r="D70" s="23"/>
-      <c r="E70" s="22"/>
-      <c r="F70" s="24"/>
-      <c r="G70" s="24"/>
-      <c r="H70" s="22"/>
+    <row r="69" spans="2:8" ht="20" x14ac:dyDescent="0.2">
+      <c r="B69" s="22" t="s">
+        <v>203</v>
+      </c>
+      <c r="C69" s="18" t="s">
+        <v>205</v>
+      </c>
+      <c r="D69" s="23"/>
+      <c r="E69" s="22"/>
+      <c r="F69" s="24"/>
+      <c r="G69" s="24"/>
+      <c r="H69" s="22"/>
+    </row>
+    <row r="70" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B70" s="15" t="s">
+        <v>87</v>
+      </c>
+      <c r="C70" s="16" t="s">
+        <v>175</v>
+      </c>
+      <c r="D70" s="16" t="s">
+        <v>176</v>
+      </c>
+      <c r="E70" s="15" t="s">
+        <v>143</v>
+      </c>
+      <c r="F70" s="17" t="s">
+        <v>170</v>
+      </c>
+      <c r="G70" s="17" t="s">
+        <v>132</v>
+      </c>
+      <c r="H70" s="15" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="71" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B71" s="15" t="s">
-        <v>88</v>
-      </c>
-      <c r="C71" s="16" t="s">
-        <v>176</v>
-      </c>
-      <c r="D71" s="16" t="s">
-        <v>177</v>
-      </c>
-      <c r="E71" s="15" t="s">
-        <v>144</v>
-      </c>
-      <c r="F71" s="17" t="s">
-        <v>171</v>
-      </c>
-      <c r="G71" s="17" t="s">
-        <v>133</v>
-      </c>
-      <c r="H71" s="15" t="s">
-        <v>89</v>
+      <c r="B71" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C71" s="13" t="s">
+        <v>222</v>
+      </c>
+      <c r="D71" s="13" t="s">
+        <v>226</v>
+      </c>
+      <c r="E71" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="F71" s="9">
+        <v>2.8</v>
+      </c>
+      <c r="G71" s="9">
+        <v>20</v>
+      </c>
+      <c r="H71" s="8" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="72" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B72" s="8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C72" s="13" t="s">
-        <v>162</v>
-      </c>
-      <c r="D72" s="13"/>
+        <v>222</v>
+      </c>
+      <c r="D72" s="13" t="s">
+        <v>223</v>
+      </c>
       <c r="E72" s="8" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="F72" s="9">
         <v>13</v>
@@ -3163,61 +3179,61 @@
         <v>100</v>
       </c>
       <c r="H72" s="8" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="73" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B73" s="8" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C73" s="13" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D73" s="13" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E73" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F73" s="9">
         <v>1</v>
       </c>
       <c r="G73" s="9"/>
       <c r="H73" s="8" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="74" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B74" s="8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C74" s="13" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D74" s="13"/>
       <c r="E74" s="8" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F74" s="9">
         <v>2</v>
       </c>
       <c r="G74" s="9"/>
       <c r="H74" s="8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="75" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B75" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C75" s="13" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D75" s="13" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E75" s="8" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F75" s="9">
         <v>1</v>
@@ -3227,37 +3243,37 @@
     </row>
     <row r="76" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B76" s="8" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C76" s="13" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D76" s="13" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E76" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F76" s="9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G76" s="9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="H76" s="8"/>
     </row>
     <row r="77" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B77" s="8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C77" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="D77" s="13" t="s">
         <v>162</v>
       </c>
-      <c r="D77" s="13" t="s">
-        <v>163</v>
-      </c>
       <c r="E77" s="8" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F77" s="9">
         <v>0</v>
@@ -3268,10 +3284,10 @@
     <row r="78" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B78" s="8"/>
       <c r="C78" s="13" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D78" s="13" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E78" s="8"/>
       <c r="F78" s="9">
@@ -3282,14 +3298,16 @@
     </row>
     <row r="79" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B79" s="5" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C79" s="11" t="s">
-        <v>206</v>
-      </c>
-      <c r="D79" s="11"/>
+        <v>221</v>
+      </c>
+      <c r="D79" s="11" t="s">
+        <v>225</v>
+      </c>
       <c r="E79" s="5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F79" s="6">
         <v>4</v>
@@ -3298,19 +3316,21 @@
         <v>20</v>
       </c>
       <c r="H79" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="80" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B80" s="5" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="C80" s="11" t="s">
-        <v>206</v>
-      </c>
-      <c r="D80" s="11"/>
+        <v>221</v>
+      </c>
+      <c r="D80" s="11" t="s">
+        <v>224</v>
+      </c>
       <c r="E80" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="F80" s="6">
         <v>20</v>
@@ -3319,40 +3339,40 @@
         <v>100</v>
       </c>
       <c r="H80" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="81" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B81" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C81" s="11" t="s">
-        <v>206</v>
+        <v>221</v>
       </c>
       <c r="D81" s="11" t="s">
-        <v>206</v>
+        <v>221</v>
       </c>
       <c r="E81" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F81" s="6">
         <v>2</v>
       </c>
       <c r="G81" s="6"/>
       <c r="H81" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="82" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B82" s="8" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C82" s="13" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D82" s="13"/>
       <c r="E82" s="8" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F82" s="9">
         <v>1</v>
@@ -3362,14 +3382,14 @@
     </row>
     <row r="83" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B83" s="8" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C83" s="13" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D83" s="13"/>
       <c r="E83" s="8" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="F83" s="9">
         <v>1</v>
@@ -3378,21 +3398,21 @@
         <v>97.5</v>
       </c>
       <c r="H83" s="8" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="84" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B84" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C84" s="13" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D84" s="13" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="E84" s="8" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F84" s="9">
         <v>1.5</v>
@@ -3402,16 +3422,16 @@
     </row>
     <row r="85" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B85" s="8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C85" s="13" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D85" s="13" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E85" s="8" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F85" s="9">
         <v>1</v>
@@ -3421,92 +3441,92 @@
     </row>
     <row r="86" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B86" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C86" s="13" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D86" s="13"/>
       <c r="E86" s="8" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F86" s="9">
         <v>1.2</v>
       </c>
       <c r="G86" s="9"/>
       <c r="H86" s="8" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="87" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B87" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C87" s="13" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D87" s="13" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E87" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F87" s="9">
         <v>1.2</v>
       </c>
       <c r="G87" s="9"/>
       <c r="H87" s="8" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="88" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B88" s="8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C88" s="13" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D88" s="13" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E88" s="8" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F88" s="9">
         <v>2.9</v>
       </c>
       <c r="G88" s="9"/>
       <c r="H88" s="8" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="89" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B89" s="8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C89" s="13" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D89" s="13" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E89" s="8" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F89" s="9">
         <v>1.2</v>
       </c>
       <c r="G89" s="9"/>
       <c r="H89" s="8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="90" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B90" s="22" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C90" s="18" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D90" s="23"/>
       <c r="E90" s="22"/>
@@ -3516,355 +3536,355 @@
     </row>
     <row r="91" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B91" s="15" t="s">
+        <v>87</v>
+      </c>
+      <c r="C91" s="16" t="s">
+        <v>175</v>
+      </c>
+      <c r="D91" s="16" t="s">
+        <v>176</v>
+      </c>
+      <c r="E91" s="15" t="s">
+        <v>143</v>
+      </c>
+      <c r="F91" s="17" t="s">
+        <v>170</v>
+      </c>
+      <c r="G91" s="17" t="s">
+        <v>132</v>
+      </c>
+      <c r="H91" s="15" t="s">
         <v>88</v>
-      </c>
-      <c r="C91" s="16" t="s">
-        <v>176</v>
-      </c>
-      <c r="D91" s="16" t="s">
-        <v>177</v>
-      </c>
-      <c r="E91" s="15" t="s">
-        <v>144</v>
-      </c>
-      <c r="F91" s="17" t="s">
-        <v>171</v>
-      </c>
-      <c r="G91" s="17" t="s">
-        <v>133</v>
-      </c>
-      <c r="H91" s="15" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="92" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B92" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C92" s="11" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D92" s="11"/>
       <c r="E92" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F92" s="6">
         <v>1.8</v>
       </c>
       <c r="G92" s="6"/>
       <c r="H92" s="5" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="93" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B93" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C93" s="11" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D93" s="11" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E93" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F93" s="6">
         <v>1.4</v>
       </c>
       <c r="G93" s="6"/>
       <c r="H93" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="94" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B94" s="5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C94" s="11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D94" s="11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E94" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F94" s="6">
         <v>10</v>
       </c>
       <c r="G94" s="6"/>
       <c r="H94" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="95" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B95" s="5" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C95" s="11" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D95" s="11" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="E95" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F95" s="6">
         <v>0.8</v>
       </c>
       <c r="G95" s="6"/>
       <c r="H95" s="5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="96" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B96" s="5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C96" s="11" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D96" s="11" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E96" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F96" s="6">
         <v>1.2</v>
       </c>
       <c r="G96" s="6"/>
       <c r="H96" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="97" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B97" s="5" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C97" s="11" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D97" s="11" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E97" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F97" s="6">
         <v>1.2</v>
       </c>
       <c r="G97" s="6"/>
       <c r="H97" s="5" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="98" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B98" s="5" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C98" s="11" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D98" s="11" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E98" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F98" s="6">
         <v>2</v>
       </c>
       <c r="G98" s="6"/>
       <c r="H98" s="5" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="99" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B99" s="8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C99" s="13" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D99" s="13"/>
       <c r="E99" s="8" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F99" s="9">
         <v>1.4</v>
       </c>
       <c r="G99" s="9"/>
       <c r="H99" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="100" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B100" s="8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C100" s="13" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D100" s="13" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E100" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F100" s="9">
         <v>1.5</v>
       </c>
       <c r="G100" s="9"/>
       <c r="H100" s="8" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="101" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B101" s="8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C101" s="13" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D101" s="13" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E101" s="8" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F101" s="9">
         <v>1</v>
       </c>
       <c r="G101" s="9"/>
       <c r="H101" s="8" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="102" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B102" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C102" s="13" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D102" s="13" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E102" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F102" s="9">
         <v>1.2</v>
       </c>
       <c r="G102" s="9"/>
       <c r="H102" s="8" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="103" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B103" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C103" s="13" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D103" s="13" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E103" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F103" s="9">
         <v>1</v>
       </c>
       <c r="G103" s="9"/>
       <c r="H103" s="8" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="104" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B104" s="8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C104" s="13" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D104" s="13" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E104" s="8" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F104" s="9">
         <v>1.4</v>
       </c>
       <c r="G104" s="9"/>
       <c r="H104" s="8" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="105" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B105" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C105" s="11" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D105" s="11"/>
       <c r="E105" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F105" s="6">
         <v>3</v>
       </c>
       <c r="G105" s="6"/>
       <c r="H105" s="5" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="106" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B106" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C106" s="11" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D106" s="11" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E106" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F106" s="6">
         <v>2</v>
       </c>
       <c r="G106" s="6"/>
       <c r="H106" s="5" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="107" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B107" s="5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C107" s="11" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D107" s="11" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E107" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F107" s="6">
         <v>1</v>
       </c>
       <c r="G107" s="6"/>
       <c r="H107" s="5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
   </sheetData>

</xml_diff>